<commit_message>
Millora del sankey (ordre dels nodes)
</commit_message>
<xml_diff>
--- a/data/sankey/sankey_nodes-at.xlsx
+++ b/data/sankey/sankey_nodes-at.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\sankey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E8ACEBC-14AC-477D-88E5-BC441E517BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6E59D8A-2CEB-4E1C-BBA2-1F645DDB53AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="86">
   <si>
     <t>source</t>
   </si>
@@ -62,9 +62,6 @@
     <t>SIL-PEL</t>
   </si>
   <si>
-    <t>LIQ-LIQ</t>
-  </si>
-  <si>
     <t>Y-120</t>
   </si>
   <si>
@@ -77,9 +74,6 @@
     <t>colector</t>
   </si>
   <si>
-    <t>GF-ass</t>
-  </si>
-  <si>
     <t>nautas</t>
   </si>
   <si>
@@ -249,6 +243,60 @@
   </si>
   <si>
     <t>rgba(255,255,0,0.4)</t>
+  </si>
+  <si>
+    <t>L-660</t>
+  </si>
+  <si>
+    <t>L-670</t>
+  </si>
+  <si>
+    <t>esquema</t>
+  </si>
+  <si>
+    <t>Y-190</t>
+  </si>
+  <si>
+    <t>Y-180</t>
+  </si>
+  <si>
+    <t>SS-3000</t>
+  </si>
+  <si>
+    <t>SS-1000</t>
+  </si>
+  <si>
+    <t>S-600</t>
+  </si>
+  <si>
+    <t>S-2100/S-2200</t>
+  </si>
+  <si>
+    <t>S-6000</t>
+  </si>
+  <si>
+    <t>SI-603</t>
+  </si>
+  <si>
+    <t>SR-601</t>
+  </si>
+  <si>
+    <t>SI-2107</t>
+  </si>
+  <si>
+    <t>SI-2207</t>
+  </si>
+  <si>
+    <t>SI-6002</t>
+  </si>
+  <si>
+    <t>SS-2200</t>
+  </si>
+  <si>
+    <t>SS-2100</t>
+  </si>
+  <si>
+    <t>GF-ASS</t>
   </si>
 </sst>
 </file>
@@ -329,14 +377,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -467,17 +514,16 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D176"/>
+  <dimension ref="A1:E178"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" style="6"/>
-    <col min="3" max="3" width="19" style="6" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="6"/>
-    <col min="5" max="16384" width="11.5546875" style="1"/>
+    <col min="1" max="1" width="18.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" style="1"/>
+    <col min="3" max="3" width="19" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.5546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" s="2" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -485,969 +531,1281 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4"/>
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D2" s="4">
-        <v>100.46507000896433</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="B3" s="4" t="s">
-        <v>13</v>
+        <v>75</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" s="4">
+        <v>65</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="4">
+        <v>203</v>
+      </c>
+      <c r="E5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="4">
+        <v>222</v>
+      </c>
+      <c r="E6" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="4">
+        <v>191</v>
+      </c>
+      <c r="E7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="4">
+        <v>205</v>
+      </c>
+      <c r="E8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="4">
+        <v>231</v>
+      </c>
+      <c r="E9" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="4">
+        <v>75</v>
+      </c>
+      <c r="E10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="4">
+        <v>72</v>
+      </c>
+      <c r="E11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D4" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="4" t="s">
+      <c r="E12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="4">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" s="4">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="4">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D10" s="4">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D11" s="4">
-        <v>56.384974069999998</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D12" s="4">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>11</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>66</v>
       </c>
       <c r="D13" s="4">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>129.48513944741836</v>
+      </c>
+      <c r="E13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="4" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D14" s="4">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>321</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D15" s="4">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>87</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="4" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="4">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>129.48513944741836</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="4">
+        <v>100.46507000896433</v>
+      </c>
+      <c r="E17" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D17" s="4">
-        <v>42.5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>8</v>
-      </c>
       <c r="C18" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D18" s="4">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="C19" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D19" s="4">
-        <v>101.8421149</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>124</v>
+      </c>
+      <c r="E19" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>66</v>
       </c>
       <c r="D20" s="4">
-        <v>32.801418630000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>32.979183040324209</v>
+      </c>
+      <c r="E20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="4" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D21" s="4">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>42.5</v>
+      </c>
+      <c r="E21" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="4" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D22" s="4">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>79.605544469999998</v>
+      </c>
+      <c r="E22" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="4" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D23" s="4">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>22.236570419999996</v>
+      </c>
+      <c r="E23" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="4" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="4">
+        <v>8.3366590708646733</v>
+      </c>
+      <c r="E24" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" s="4">
+        <v>28.217898310000002</v>
+      </c>
+      <c r="E25" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D26" s="4">
+        <v>20.000000000000004</v>
+      </c>
+      <c r="E26" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" s="4">
+        <v>41</v>
+      </c>
+      <c r="E27" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D25" s="4">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="4" t="s">
+      <c r="E28" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D26" s="4">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="4">
-        <v>30.4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D28" s="4">
-        <v>79.605544469999998</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>30</v>
-      </c>
       <c r="C29" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D29" s="4">
-        <v>22.236570419999996</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+      <c r="E29" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D30" s="4">
-        <v>20.000000000000004</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>75</v>
+      </c>
+      <c r="E30" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D31" s="4">
         <v>10.190084069999997</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="E31" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B32" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="4">
+        <v>32.801418630000001</v>
+      </c>
+      <c r="E32" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" s="4">
+        <v>67</v>
+      </c>
+      <c r="E33" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" s="4">
+        <v>44</v>
+      </c>
+      <c r="E34" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D35" s="4">
+        <v>47</v>
+      </c>
+      <c r="E35" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36" s="4">
+        <v>150</v>
+      </c>
+      <c r="E36" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D37" s="4">
+        <v>23.5</v>
+      </c>
+      <c r="E37" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D32" s="4">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D33" s="4">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D34" s="4">
-        <v>23.5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D35" s="4">
-        <v>13.601897040000001</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D36" s="4">
+      <c r="C38" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D38" s="4">
         <v>17.5</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A37" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D37" s="4">
-        <v>15.34166403</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D38" s="4">
-        <v>13.89928536</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="E38" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A39" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D39" s="4">
-        <v>25.380859569999998</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>56.384974069999998</v>
+      </c>
+      <c r="E39" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A40" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>46</v>
+        <v>6</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D40" s="4">
-        <v>17.134670450000002</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>30.4</v>
+      </c>
+      <c r="E40" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A41" s="4" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D41" s="4">
-        <v>28.217898310000002</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>13.8940359441001</v>
+      </c>
+      <c r="E41" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A42" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>66</v>
       </c>
       <c r="D42" s="4">
-        <v>10.822828879999999</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>1</v>
+      </c>
+      <c r="E42" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A43" s="4" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D43" s="4">
-        <v>8.1686317729999995</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>13.601897040000001</v>
+      </c>
+      <c r="E43" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A44" s="4" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D44" s="4">
         <v>10.822828879999999</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="E44" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A45" s="4" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="C45" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D45" s="4">
+        <v>32.979183040324209</v>
+      </c>
+      <c r="E45" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A46" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D46" s="4"/>
+      <c r="E46" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A47" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D47" s="4"/>
+      <c r="E47" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A48" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C48" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D45" s="4">
-        <v>1.17621229</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A46" s="4" t="s">
+      <c r="D48" s="4">
+        <v>3.8707563084879837</v>
+      </c>
+      <c r="E48" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A49" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D49" s="4">
+        <v>5.0590982872275125</v>
+      </c>
+      <c r="E49" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A50" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D50" s="4">
+        <v>8.1686317729999995</v>
+      </c>
+      <c r="E50" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A51" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D51" s="4">
+        <v>32.979183040324209</v>
+      </c>
+      <c r="E51" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A52" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D46" s="4">
-        <v>129.48513944741836</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A47" s="4" t="s">
+      <c r="B52" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D52" s="4"/>
+      <c r="E52" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A53" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D47" s="4">
-        <v>129.48513944741836</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A48" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D48" s="4">
-        <v>32.979183040324209</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A49" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D49" s="4">
-        <v>19.43128149161133</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A50" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D50" s="4">
-        <v>19.43128149161133</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A51" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D51" s="4">
-        <v>8.3366590708646733</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A52" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D52" s="4">
-        <v>8.3366590708646733</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A53" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="B53" s="4" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D53" s="4">
-        <v>8.3366590708646733</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>65</v>
+      </c>
+      <c r="D53" s="4"/>
+      <c r="E53" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A54" s="4" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>63</v>
+        <v>34</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D54" s="4">
-        <v>8.3366590708646733</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>10.822828879999999</v>
+      </c>
+      <c r="E54" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A55" s="4" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D55" s="4">
         <v>8.3366590708646733</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="E55" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="B56" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D56" s="4">
+        <v>101.8421149</v>
+      </c>
+      <c r="E56" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A57" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D57" s="4">
+        <v>28</v>
+      </c>
+      <c r="E57" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A58" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D58" s="4"/>
+      <c r="E58" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A59" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D59" s="4"/>
+      <c r="E59" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A60" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D60" s="4"/>
+      <c r="E60" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A61" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D61" s="4"/>
+      <c r="E61" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A62" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D62" s="4"/>
+      <c r="E62" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A63" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A64" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A65" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D65" s="4">
+        <v>8.3366590708646733</v>
+      </c>
+      <c r="E65" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A66" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D66" s="4">
+        <v>8.3366590708646733</v>
+      </c>
+      <c r="E66" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A67" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D67" s="4">
+        <v>15.34166403</v>
+      </c>
+      <c r="E67" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A68" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D68" s="4">
+        <v>13.89928536</v>
+      </c>
+      <c r="E68" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A69" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D69" s="4">
+        <v>1.17621229</v>
+      </c>
+      <c r="E69" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A70" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D70" s="4">
+        <v>19.43128149161133</v>
+      </c>
+      <c r="E70" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A71" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D71" s="4">
+        <v>19.43128149161133</v>
+      </c>
+      <c r="E71" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A72" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D72" s="4">
+        <v>8.3366590708646733</v>
+      </c>
+      <c r="E72" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A73" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D73" s="4">
+        <v>0</v>
+      </c>
+      <c r="E73" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A74" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D74" s="4">
+        <v>0</v>
+      </c>
+      <c r="E74" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A75" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B75" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C56" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D56" s="4">
-        <v>8.3366590708646733</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A57" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B57" s="4" t="s">
+      <c r="C75" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D75" s="4">
+        <v>17.134670450000002</v>
+      </c>
+      <c r="E75" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A76" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B76" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C57" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D57" s="4">
-        <v>8.3366590708646733</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A58" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B58" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D58" s="4">
-        <v>5.0590982872275125</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A59" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D59" s="4">
-        <v>3.8707563084879837</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A60" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D60" s="4">
-        <v>32.979183040324209</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A61" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D61" s="4">
-        <v>32.979183040324209</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A62" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D62" s="4">
-        <v>13.8940359441001</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A63" s="5"/>
-      <c r="B63" s="5"/>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-    </row>
-    <row r="64" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A64" s="5"/>
-      <c r="B64" s="5"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="5"/>
-    </row>
-    <row r="65" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A65" s="5"/>
-      <c r="B65" s="5"/>
-      <c r="C65" s="5"/>
-      <c r="D65" s="5"/>
-    </row>
-    <row r="66" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A66" s="5"/>
-      <c r="B66" s="5"/>
-      <c r="C66" s="5"/>
-      <c r="D66" s="5"/>
-    </row>
-    <row r="67" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A67" s="5"/>
-      <c r="B67" s="5"/>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-    </row>
-    <row r="68" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A68" s="5"/>
-      <c r="B68" s="5"/>
-      <c r="C68" s="5"/>
-      <c r="D68" s="5"/>
-    </row>
-    <row r="69" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A69" s="5"/>
-      <c r="B69" s="5"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="5"/>
-    </row>
-    <row r="70" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A70" s="5"/>
-      <c r="B70" s="5"/>
-      <c r="C70" s="5"/>
-      <c r="D70" s="5"/>
-    </row>
-    <row r="71" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A71" s="5"/>
-      <c r="B71" s="5"/>
-      <c r="C71" s="5"/>
-      <c r="D71" s="5"/>
-    </row>
-    <row r="72" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A72" s="5"/>
-      <c r="B72" s="5"/>
-      <c r="C72" s="5"/>
-      <c r="D72" s="5"/>
-    </row>
-    <row r="73" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A73" s="5"/>
-      <c r="B73" s="5"/>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-    </row>
-    <row r="74" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A74" s="5"/>
-      <c r="B74" s="5"/>
-      <c r="C74" s="5"/>
-      <c r="D74" s="5"/>
-    </row>
-    <row r="75" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A75" s="5"/>
-      <c r="B75" s="5"/>
-      <c r="C75" s="5"/>
-      <c r="D75" s="5"/>
-    </row>
-    <row r="76" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A76" s="5"/>
-      <c r="B76" s="5"/>
-      <c r="C76" s="5"/>
-      <c r="D76" s="5"/>
-    </row>
-    <row r="77" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="C76" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D76" s="4">
+        <v>25.380859569999998</v>
+      </c>
+      <c r="E76" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A77" s="5"/>
       <c r="B77" s="5"/>
       <c r="C77" s="5"/>
       <c r="D77" s="5"/>
     </row>
-    <row r="78" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A78" s="5"/>
       <c r="B78" s="5"/>
       <c r="C78" s="5"/>
       <c r="D78" s="5"/>
     </row>
-    <row r="79" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A79" s="5"/>
       <c r="B79" s="5"/>
       <c r="C79" s="5"/>
       <c r="D79" s="5"/>
     </row>
-    <row r="80" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A80" s="5"/>
       <c r="B80" s="5"/>
       <c r="C80" s="5"/>
@@ -2029,10 +2387,22 @@
       <c r="C176" s="5"/>
       <c r="D176" s="5"/>
     </row>
+    <row r="177" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A177" s="5"/>
+      <c r="B177" s="5"/>
+      <c r="C177" s="5"/>
+      <c r="D177" s="5"/>
+    </row>
+    <row r="178" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A178" s="5"/>
+      <c r="B178" s="5"/>
+      <c r="C178" s="5"/>
+      <c r="D178" s="5"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D72">
-      <sortCondition ref="C1"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D77">
+      <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Millores a punts de mesura i afegir R-150
</commit_message>
<xml_diff>
--- a/data/sankey/sankey_nodes-at.xlsx
+++ b/data/sankey/sankey_nodes-at.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\sankey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8880D3B-5CD7-439D-85EC-8D7586C9A6BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{955A0B3E-E89C-4758-A9C0-CBCDEE883CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="101">
   <si>
     <t>source</t>
   </si>
@@ -336,6 +336,12 @@
   </si>
   <si>
     <t>S-60021</t>
+  </si>
+  <si>
+    <t>R-150</t>
+  </si>
+  <si>
+    <t>rgba(255,255, 0, 0.4)</t>
   </si>
 </sst>
 </file>
@@ -553,7 +559,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E179"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="18.88671875" style="1" customWidth="1"/>
@@ -754,7 +760,7 @@
         <v>65</v>
       </c>
       <c r="D12" s="4">
-        <f>SUM(D77:D79)</f>
+        <f>SUM(D78:D80)</f>
         <v>78.997951654825172</v>
       </c>
       <c r="E12" s="1">
@@ -857,7 +863,7 @@
         <v>65</v>
       </c>
       <c r="D18" s="4">
-        <f>SUM(D84:D85)</f>
+        <f>SUM(D85:D86)</f>
         <v>15.944518911578967</v>
       </c>
       <c r="E18" s="1">
@@ -1325,15 +1331,17 @@
     </row>
     <row r="46" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A46" s="4" t="s">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>72</v>
+        <v>99</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D46" s="4"/>
+        <v>100</v>
+      </c>
+      <c r="D46" s="4">
+        <v>18.5</v>
+      </c>
       <c r="E46" s="1">
         <v>1</v>
       </c>
@@ -1343,7 +1351,7 @@
         <v>85</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>65</v>
@@ -1355,17 +1363,15 @@
     </row>
     <row r="48" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A48" s="4" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>36</v>
+        <v>71</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D48" s="4">
-        <v>3.8707563084879837</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="D48" s="4"/>
       <c r="E48" s="1">
         <v>1</v>
       </c>
@@ -1375,13 +1381,13 @@
         <v>68</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>66</v>
       </c>
       <c r="D49" s="4">
-        <v>5.0590982872275125</v>
+        <v>3.8707563084879837</v>
       </c>
       <c r="E49" s="1">
         <v>1</v>
@@ -1389,16 +1395,16 @@
     </row>
     <row r="50" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A50" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D50" s="4">
-        <v>8.1686317729999995</v>
+        <v>5.0590982872275125</v>
       </c>
       <c r="E50" s="1">
         <v>1</v>
@@ -1409,13 +1415,13 @@
         <v>69</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D51" s="4">
-        <v>32.979183040324209</v>
+        <v>8.1686317729999995</v>
       </c>
       <c r="E51" s="1">
         <v>1</v>
@@ -1423,15 +1429,17 @@
     </row>
     <row r="52" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A52" s="4" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D52" s="4"/>
+        <v>66</v>
+      </c>
+      <c r="D52" s="4">
+        <v>32.979183040324209</v>
+      </c>
       <c r="E52" s="1">
         <v>1</v>
       </c>
@@ -1441,7 +1449,7 @@
         <v>11</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>65</v>
@@ -1453,17 +1461,15 @@
     </row>
     <row r="54" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A54" s="4" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="D54" s="4">
-        <v>10.822828879999999</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="D54" s="4"/>
       <c r="E54" s="1">
         <v>1</v>
       </c>
@@ -1473,13 +1479,13 @@
         <v>21</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D55" s="4">
-        <v>8.3366590708646733</v>
+        <v>10.822828879999999</v>
       </c>
       <c r="E55" s="1">
         <v>1</v>
@@ -1487,16 +1493,16 @@
     </row>
     <row r="56" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A56" s="4" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D56" s="4">
-        <v>101.8421149</v>
+        <v>8.3366590708646733</v>
       </c>
       <c r="E56" s="1">
         <v>1</v>
@@ -1507,13 +1513,13 @@
         <v>5</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>64</v>
       </c>
       <c r="D57" s="4">
-        <v>28</v>
+        <v>101.8421149</v>
       </c>
       <c r="E57" s="1">
         <v>1</v>
@@ -1521,15 +1527,17 @@
     </row>
     <row r="58" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A58" s="4" t="s">
-        <v>76</v>
+        <v>5</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D58" s="4"/>
+        <v>64</v>
+      </c>
+      <c r="D58" s="4">
+        <v>28</v>
+      </c>
       <c r="E58" s="1">
         <v>1</v>
       </c>
@@ -1539,7 +1547,7 @@
         <v>76</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>65</v>
@@ -1554,7 +1562,7 @@
         <v>76</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>65</v>
@@ -1569,7 +1577,7 @@
         <v>76</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>65</v>
@@ -1581,10 +1589,10 @@
     </row>
     <row r="62" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A62" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>65</v>
@@ -1599,22 +1607,22 @@
         <v>75</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D63" s="4"/>
-      <c r="E63" s="4">
+      <c r="E63" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A64" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>65</v>
@@ -1626,17 +1634,15 @@
     </row>
     <row r="65" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A65" s="4" t="s">
-        <v>6</v>
+        <v>77</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="D65" s="4">
-        <v>8.3366590708646733</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="D65" s="4"/>
       <c r="E65" s="4">
         <v>1</v>
       </c>
@@ -1646,7 +1652,7 @@
         <v>6</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>66</v>
@@ -1663,13 +1669,13 @@
         <v>6</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D67" s="4">
-        <v>15.34166403</v>
+        <v>8.3366590708646733</v>
       </c>
       <c r="E67" s="4">
         <v>1</v>
@@ -1680,13 +1686,13 @@
         <v>6</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>64</v>
       </c>
       <c r="D68" s="4">
-        <v>13.89928536</v>
+        <v>15.34166403</v>
       </c>
       <c r="E68" s="4">
         <v>1</v>
@@ -1697,13 +1703,13 @@
         <v>6</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>64</v>
       </c>
       <c r="D69" s="4">
-        <v>1.17621229</v>
+        <v>13.89928536</v>
       </c>
       <c r="E69" s="4">
         <v>1</v>
@@ -1711,16 +1717,16 @@
     </row>
     <row r="70" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A70" s="4" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D70" s="4">
-        <v>19.43128149161133</v>
+        <v>1.17621229</v>
       </c>
       <c r="E70" s="4">
         <v>1</v>
@@ -1728,10 +1734,10 @@
     </row>
     <row r="71" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A71" s="4" t="s">
-        <v>22</v>
+        <v>56</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>66</v>
@@ -1748,13 +1754,13 @@
         <v>22</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>66</v>
       </c>
       <c r="D72" s="4">
-        <v>8.3366590708646733</v>
+        <v>19.43128149161133</v>
       </c>
       <c r="E72" s="4">
         <v>1</v>
@@ -1762,16 +1768,16 @@
     </row>
     <row r="73" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A73" s="4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>66</v>
       </c>
       <c r="D73" s="4">
-        <v>0</v>
+        <v>8.3366590708646733</v>
       </c>
       <c r="E73" s="4">
         <v>1</v>
@@ -1782,7 +1788,7 @@
         <v>14</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>66</v>
@@ -1799,13 +1805,13 @@
         <v>14</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D75" s="4">
-        <v>17.134670450000002</v>
+        <v>0</v>
       </c>
       <c r="E75" s="4">
         <v>1</v>
@@ -1816,13 +1822,13 @@
         <v>14</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>64</v>
       </c>
       <c r="D76" s="4">
-        <v>25.380859569999998</v>
+        <v>17.134670450000002</v>
       </c>
       <c r="E76" s="4">
         <v>1</v>
@@ -1830,17 +1836,16 @@
     </row>
     <row r="77" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A77" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D77" s="4">
-        <f>SUM(D89:D91)</f>
-        <v>34.817325760346947</v>
+        <v>25.380859569999998</v>
       </c>
       <c r="E77" s="4">
         <v>1</v>
@@ -1851,14 +1856,14 @@
         <v>12</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D78" s="4">
-        <f>D86</f>
-        <v>13.422420054943197</v>
+        <f>SUM(D90:D92)</f>
+        <v>34.817325760346947</v>
       </c>
       <c r="E78" s="4">
         <v>1</v>
@@ -1869,14 +1874,14 @@
         <v>12</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D79" s="4">
-        <f>D92</f>
-        <v>30.75820583953503</v>
+        <f>D87</f>
+        <v>13.422420054943197</v>
       </c>
       <c r="E79" s="4">
         <v>1</v>
@@ -1884,16 +1889,17 @@
     </row>
     <row r="80" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A80" s="4" t="s">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D80" s="4">
-        <v>13.422420054943197</v>
+        <f>D93</f>
+        <v>30.75820583953503</v>
       </c>
       <c r="E80" s="4">
         <v>1</v>
@@ -1904,7 +1910,7 @@
         <v>85</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>65</v>
@@ -1921,7 +1927,7 @@
         <v>85</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>65</v>
@@ -1938,7 +1944,7 @@
         <v>85</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>65</v>
@@ -1952,16 +1958,16 @@
     </row>
     <row r="84" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A84" s="4" t="s">
-        <v>11</v>
+        <v>85</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D84" s="4">
-        <v>7.9722594557894837</v>
+        <v>13.422420054943197</v>
       </c>
       <c r="E84" s="4">
         <v>1</v>
@@ -1972,7 +1978,7 @@
         <v>11</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>65</v>
@@ -1986,16 +1992,16 @@
     </row>
     <row r="86" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A86" s="4" t="s">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D86" s="4">
-        <v>13.422420054943197</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="E86" s="4">
         <v>1</v>
@@ -2003,10 +2009,10 @@
     </row>
     <row r="87" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A87" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>65</v>
@@ -2023,13 +2029,13 @@
         <v>76</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D88" s="4">
-        <v>7.9722594557894837</v>
+        <v>13.422420054943197</v>
       </c>
       <c r="E88" s="4">
         <v>1</v>
@@ -2040,13 +2046,13 @@
         <v>76</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D89" s="4">
-        <v>18.872806848767983</v>
+        <v>7.9722594557894837</v>
       </c>
       <c r="E89" s="4">
         <v>1</v>
@@ -2057,13 +2063,13 @@
         <v>76</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D90" s="4">
-        <v>7.9722594557894837</v>
+        <v>18.872806848767983</v>
       </c>
       <c r="E90" s="4">
         <v>1</v>
@@ -2074,7 +2080,7 @@
         <v>76</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>65</v>
@@ -2088,26 +2094,37 @@
     </row>
     <row r="92" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A92" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D92" s="4">
+        <v>7.9722594557894837</v>
+      </c>
+      <c r="E92" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A93" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="B92" s="4" t="s">
+      <c r="B93" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C92" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D92" s="4">
+      <c r="C93" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D93" s="4">
         <v>30.75820583953503</v>
       </c>
-      <c r="E92" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A93" s="5"/>
-      <c r="B93" s="5"/>
-      <c r="C93" s="5"/>
-      <c r="D93" s="5"/>
+      <c r="E93" s="4">
+        <v>1</v>
+      </c>
     </row>
     <row r="94" spans="1:5" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A94" s="5"/>
@@ -2624,6 +2641,12 @@
       <c r="B179" s="5"/>
       <c r="C179" s="5"/>
       <c r="D179" s="5"/>
+    </row>
+    <row r="180" spans="1:4" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A180" s="5"/>
+      <c r="B180" s="5"/>
+      <c r="C180" s="5"/>
+      <c r="D180" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>